<commit_message>
Geração dos dados de teste funcionando - necessário verificar ainda
</commit_message>
<xml_diff>
--- a/Faturados.xlsx
+++ b/Faturados.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="760" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="792" uniqueCount="208">
   <si>
     <t>Código Produto</t>
   </si>
@@ -172,6 +172,9 @@
     <t>PROD400003</t>
   </si>
   <si>
+    <t>PROD400004</t>
+  </si>
+  <si>
     <t>PROD500001</t>
   </si>
   <si>
@@ -286,6 +289,9 @@
     <t>Produto de Teste - Processo 400003</t>
   </si>
   <si>
+    <t>Produto de Teste - Processo 400004</t>
+  </si>
+  <si>
     <t>Produto de Teste - Processo 500001</t>
   </si>
   <si>
@@ -406,6 +412,9 @@
     <t>400003</t>
   </si>
   <si>
+    <t>400004</t>
+  </si>
+  <si>
     <t>500001</t>
   </si>
   <si>
@@ -520,22 +529,28 @@
     <t>32000</t>
   </si>
   <si>
-    <t>Alessandro Cappi</t>
-  </si>
-  <si>
-    <t>André Caramello</t>
-  </si>
-  <si>
-    <t>Andrey Andrade</t>
-  </si>
-  <si>
-    <t>Mateus Machado</t>
-  </si>
-  <si>
-    <t>André Camargo</t>
-  </si>
-  <si>
-    <t>Leonardo Carmo</t>
+    <t>ANDREY.ANDRADE</t>
+  </si>
+  <si>
+    <t>DENER.MARTINS</t>
+  </si>
+  <si>
+    <t>SAMANTA</t>
+  </si>
+  <si>
+    <t>JULIANO</t>
+  </si>
+  <si>
+    <t>ROSANA.MARTINS</t>
+  </si>
+  <si>
+    <t>ANDRÉ LUIS GONCALVES CAMARGO</t>
+  </si>
+  <si>
+    <t>MATEUS BORRO MACHADO</t>
+  </si>
+  <si>
+    <t>LEONARDO DO CARMO</t>
   </si>
   <si>
     <t>Industrial</t>
@@ -574,21 +589,27 @@
     <t>ISCO</t>
   </si>
   <si>
+    <t>MicroClip</t>
+  </si>
+  <si>
+    <t>E3 Point</t>
+  </si>
+  <si>
+    <t>EXO</t>
+  </si>
+  <si>
     <t>QED</t>
   </si>
   <si>
-    <t>MicroClip</t>
-  </si>
-  <si>
-    <t>EXO</t>
+    <t>Panther</t>
+  </si>
+  <si>
+    <t>YSI</t>
   </si>
   <si>
     <t>Thermo</t>
   </si>
   <si>
-    <t>YSI</t>
-  </si>
-  <si>
     <t>Analisador Fixo</t>
   </si>
   <si>
@@ -598,13 +619,16 @@
     <t>Equipamento Amostragem</t>
   </si>
   <si>
+    <t>Detector Portátil</t>
+  </si>
+  <si>
+    <t>Detector Fixo</t>
+  </si>
+  <si>
+    <t>Sonda Multiparâmetros</t>
+  </si>
+  <si>
     <t>Sistema Remediação</t>
-  </si>
-  <si>
-    <t>Detector Portátil</t>
-  </si>
-  <si>
-    <t>Sonda Multiparâmetros</t>
   </si>
   <si>
     <t>SSO</t>
@@ -975,7 +999,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T44"/>
+  <dimension ref="A1:T46"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:20">
@@ -1045,55 +1069,52 @@
         <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F2" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G2" s="2">
         <v>45894</v>
       </c>
       <c r="H2" t="s">
-        <v>137</v>
-      </c>
-      <c r="I2" t="s">
-        <v>168</v>
+        <v>140</v>
       </c>
       <c r="L2" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M2" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N2" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O2" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P2" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q2" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R2" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="S2" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="T2" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -1101,55 +1122,52 @@
         <v>21</v>
       </c>
       <c r="B3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F3" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G3" s="2">
         <v>45889</v>
       </c>
       <c r="H3" t="s">
-        <v>138</v>
-      </c>
-      <c r="I3" t="s">
-        <v>169</v>
+        <v>141</v>
       </c>
       <c r="L3" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M3" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N3" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O3" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P3" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q3" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R3" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="S3" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="T3" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -1157,55 +1175,52 @@
         <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C4" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D4" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E4" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F4" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G4" s="2">
         <v>45884</v>
       </c>
       <c r="H4" t="s">
-        <v>139</v>
-      </c>
-      <c r="I4" t="s">
-        <v>168</v>
+        <v>142</v>
       </c>
       <c r="L4" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M4" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N4" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O4" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P4" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q4" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R4" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="S4" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="T4" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
     </row>
     <row r="5" spans="1:20">
@@ -1213,55 +1228,58 @@
         <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D5" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F5" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G5" s="2">
         <v>45884</v>
       </c>
       <c r="H5" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="I5" t="s">
-        <v>170</v>
+        <v>171</v>
+      </c>
+      <c r="J5" t="s">
+        <v>176</v>
       </c>
       <c r="L5" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M5" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N5" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O5" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P5" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q5" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R5" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="S5" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="T5" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
     </row>
     <row r="6" spans="1:20">
@@ -1269,58 +1287,58 @@
         <v>24</v>
       </c>
       <c r="B6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E6" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F6" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G6" s="2">
         <v>45887</v>
       </c>
       <c r="H6" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="I6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="J6" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="L6" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M6" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N6" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O6" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P6" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q6" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R6" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="S6" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="T6" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
     </row>
     <row r="7" spans="1:20">
@@ -1328,55 +1346,55 @@
         <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D7" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E7" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F7" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G7" s="2">
         <v>45889</v>
       </c>
       <c r="H7" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="J7" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="L7" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M7" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N7" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O7" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P7" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q7" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R7" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="S7" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="T7" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
     </row>
     <row r="8" spans="1:20">
@@ -1384,55 +1402,55 @@
         <v>26</v>
       </c>
       <c r="B8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D8" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E8" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F8" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G8" s="2">
         <v>45891</v>
       </c>
       <c r="H8" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="I8" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="L8" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M8" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N8" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O8" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P8" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q8" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R8" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="S8" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="T8" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
     </row>
     <row r="9" spans="1:20">
@@ -1440,58 +1458,58 @@
         <v>27</v>
       </c>
       <c r="B9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C9" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D9" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E9" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F9" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G9" s="2">
         <v>45894</v>
       </c>
       <c r="H9" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="I9" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="J9" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="L9" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M9" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N9" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O9" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q9" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R9" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="S9" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="T9" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
     </row>
     <row r="10" spans="1:20">
@@ -1499,55 +1517,58 @@
         <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C10" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D10" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E10" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F10" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G10" s="2">
         <v>45897</v>
       </c>
       <c r="H10" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="I10" t="s">
-        <v>170</v>
+        <v>171</v>
+      </c>
+      <c r="J10" t="s">
+        <v>176</v>
       </c>
       <c r="L10" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M10" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N10" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O10" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P10" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q10" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R10" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="S10" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="T10" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
     </row>
     <row r="11" spans="1:20">
@@ -1555,55 +1576,58 @@
         <v>28</v>
       </c>
       <c r="B11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C11" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D11" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E11" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F11" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G11" s="2">
         <v>45897</v>
       </c>
       <c r="H11" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="I11" t="s">
         <v>171</v>
       </c>
+      <c r="J11" t="s">
+        <v>176</v>
+      </c>
       <c r="L11" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M11" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N11" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O11" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P11" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q11" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R11" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="S11" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="T11" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
     </row>
     <row r="12" spans="1:20">
@@ -1611,55 +1635,52 @@
         <v>29</v>
       </c>
       <c r="B12" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C12" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D12" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E12" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F12" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G12" s="2">
         <v>45885</v>
       </c>
       <c r="H12" t="s">
-        <v>143</v>
-      </c>
-      <c r="I12" t="s">
-        <v>170</v>
+        <v>146</v>
       </c>
       <c r="L12" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M12" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N12" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O12" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P12" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q12" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="R12" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="S12" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="T12" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
     </row>
     <row r="13" spans="1:20">
@@ -1667,55 +1688,58 @@
         <v>30</v>
       </c>
       <c r="B13" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C13" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D13" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E13" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F13" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G13" s="2">
         <v>45886</v>
       </c>
       <c r="H13" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="I13" t="s">
-        <v>170</v>
+        <v>173</v>
+      </c>
+      <c r="J13" t="s">
+        <v>176</v>
       </c>
       <c r="L13" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M13" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N13" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O13" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P13" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q13" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R13" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="S13" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="T13" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
     </row>
     <row r="14" spans="1:20">
@@ -1723,55 +1747,55 @@
         <v>31</v>
       </c>
       <c r="B14" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C14" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D14" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E14" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F14" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G14" s="2">
         <v>45887</v>
       </c>
       <c r="H14" t="s">
-        <v>145</v>
-      </c>
-      <c r="I14" t="s">
-        <v>170</v>
+        <v>148</v>
+      </c>
+      <c r="J14" t="s">
+        <v>177</v>
       </c>
       <c r="L14" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M14" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N14" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O14" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P14" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q14" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="R14" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
       <c r="S14" t="s">
-        <v>191</v>
+        <v>203</v>
       </c>
       <c r="T14" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
     </row>
     <row r="15" spans="1:20">
@@ -1779,55 +1803,58 @@
         <v>32</v>
       </c>
       <c r="B15" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C15" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D15" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E15" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="F15" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G15" s="2">
         <v>45888</v>
       </c>
       <c r="H15" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="I15" t="s">
-        <v>170</v>
+        <v>174</v>
+      </c>
+      <c r="J15" t="s">
+        <v>177</v>
       </c>
       <c r="L15" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M15" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N15" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O15" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P15" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q15" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="R15" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="S15" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="T15" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
     </row>
     <row r="16" spans="1:20">
@@ -1835,55 +1862,52 @@
         <v>33</v>
       </c>
       <c r="B16" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C16" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D16" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E16" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F16" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G16" s="2">
         <v>45889</v>
       </c>
       <c r="H16" t="s">
-        <v>147</v>
-      </c>
-      <c r="I16" t="s">
-        <v>170</v>
+        <v>150</v>
       </c>
       <c r="L16" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M16" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N16" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O16" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P16" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q16" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="R16" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="S16" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
       <c r="T16" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
     </row>
     <row r="17" spans="1:20">
@@ -1891,55 +1915,58 @@
         <v>34</v>
       </c>
       <c r="B17" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C17" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D17" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E17" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F17" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G17" s="2">
         <v>45890</v>
       </c>
       <c r="H17" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="I17" t="s">
-        <v>170</v>
+        <v>172</v>
+      </c>
+      <c r="J17" t="s">
+        <v>177</v>
       </c>
       <c r="L17" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M17" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N17" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O17" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P17" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q17" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R17" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="S17" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="T17" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
     </row>
     <row r="18" spans="1:20">
@@ -1947,55 +1974,55 @@
         <v>35</v>
       </c>
       <c r="B18" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C18" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D18" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E18" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F18" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G18" s="2">
         <v>45891</v>
       </c>
       <c r="H18" t="s">
-        <v>149</v>
-      </c>
-      <c r="I18" t="s">
-        <v>170</v>
+        <v>152</v>
+      </c>
+      <c r="J18" t="s">
+        <v>178</v>
       </c>
       <c r="L18" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M18" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N18" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O18" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P18" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q18" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="R18" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="S18" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="T18" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
     </row>
     <row r="19" spans="1:20">
@@ -2003,55 +2030,58 @@
         <v>36</v>
       </c>
       <c r="B19" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C19" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D19" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E19" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F19" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G19" s="2">
         <v>45892</v>
       </c>
       <c r="H19" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="I19" t="s">
-        <v>170</v>
+        <v>175</v>
+      </c>
+      <c r="J19" t="s">
+        <v>176</v>
       </c>
       <c r="L19" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M19" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N19" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O19" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P19" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q19" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="R19" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="S19" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="T19" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
     </row>
     <row r="20" spans="1:20">
@@ -2059,55 +2089,52 @@
         <v>37</v>
       </c>
       <c r="B20" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C20" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D20" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E20" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F20" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G20" s="2">
         <v>45893</v>
       </c>
       <c r="H20" t="s">
-        <v>151</v>
-      </c>
-      <c r="I20" t="s">
-        <v>170</v>
+        <v>154</v>
       </c>
       <c r="L20" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M20" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N20" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O20" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P20" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q20" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="R20" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
       <c r="S20" t="s">
-        <v>191</v>
+        <v>203</v>
       </c>
       <c r="T20" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
     </row>
     <row r="21" spans="1:20">
@@ -2115,55 +2142,58 @@
         <v>38</v>
       </c>
       <c r="B21" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C21" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D21" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E21" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F21" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G21" s="2">
         <v>45894</v>
       </c>
       <c r="H21" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="I21" t="s">
-        <v>170</v>
+        <v>171</v>
+      </c>
+      <c r="J21" t="s">
+        <v>176</v>
       </c>
       <c r="L21" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M21" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N21" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O21" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P21" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q21" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R21" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="S21" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="T21" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
     </row>
     <row r="22" spans="1:20">
@@ -2171,55 +2201,55 @@
         <v>39</v>
       </c>
       <c r="B22" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C22" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D22" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E22" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F22" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G22" s="2">
         <v>45895</v>
       </c>
       <c r="H22" t="s">
-        <v>152</v>
-      </c>
-      <c r="I22" t="s">
-        <v>170</v>
+        <v>155</v>
+      </c>
+      <c r="J22" t="s">
+        <v>178</v>
       </c>
       <c r="L22" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M22" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N22" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O22" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P22" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q22" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="R22" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="S22" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
       <c r="T22" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
     </row>
     <row r="23" spans="1:20">
@@ -2227,55 +2257,58 @@
         <v>40</v>
       </c>
       <c r="B23" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C23" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D23" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E23" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F23" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G23" s="2">
         <v>45896</v>
       </c>
       <c r="H23" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="I23" t="s">
-        <v>170</v>
+        <v>173</v>
+      </c>
+      <c r="J23" t="s">
+        <v>177</v>
       </c>
       <c r="L23" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M23" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N23" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O23" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P23" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q23" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="R23" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="S23" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="T23" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
     </row>
     <row r="24" spans="1:20">
@@ -2283,55 +2316,52 @@
         <v>41</v>
       </c>
       <c r="B24" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C24" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D24" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E24" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F24" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G24" s="2">
         <v>45897</v>
       </c>
       <c r="H24" t="s">
-        <v>154</v>
-      </c>
-      <c r="I24" t="s">
-        <v>170</v>
+        <v>157</v>
       </c>
       <c r="L24" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M24" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N24" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O24" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P24" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q24" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="R24" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="S24" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="T24" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
     </row>
     <row r="25" spans="1:20">
@@ -2339,55 +2369,58 @@
         <v>42</v>
       </c>
       <c r="B25" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C25" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D25" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E25" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F25" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G25" s="2">
         <v>45898</v>
       </c>
       <c r="H25" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="I25" t="s">
-        <v>170</v>
+        <v>174</v>
+      </c>
+      <c r="J25" t="s">
+        <v>176</v>
       </c>
       <c r="L25" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M25" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N25" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O25" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P25" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q25" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R25" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="S25" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="T25" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
     </row>
     <row r="26" spans="1:20">
@@ -2395,55 +2428,55 @@
         <v>43</v>
       </c>
       <c r="B26" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C26" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D26" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E26" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F26" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G26" s="2">
         <v>45874</v>
       </c>
       <c r="H26" t="s">
-        <v>156</v>
-      </c>
-      <c r="I26" t="s">
-        <v>170</v>
+        <v>159</v>
+      </c>
+      <c r="J26" t="s">
+        <v>177</v>
       </c>
       <c r="L26" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M26" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N26" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O26" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P26" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q26" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="R26" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
       <c r="S26" t="s">
-        <v>191</v>
+        <v>203</v>
       </c>
       <c r="T26" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
     </row>
     <row r="27" spans="1:20">
@@ -2451,55 +2484,58 @@
         <v>44</v>
       </c>
       <c r="B27" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C27" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D27" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E27" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F27" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G27" s="2">
         <v>45875</v>
       </c>
       <c r="H27" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="I27" t="s">
-        <v>170</v>
+        <v>172</v>
+      </c>
+      <c r="J27" t="s">
+        <v>177</v>
       </c>
       <c r="L27" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M27" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N27" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O27" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P27" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q27" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="R27" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="S27" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="T27" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
     </row>
     <row r="28" spans="1:20">
@@ -2507,55 +2543,52 @@
         <v>45</v>
       </c>
       <c r="B28" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C28" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D28" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E28" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F28" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G28" s="2">
         <v>45876</v>
       </c>
       <c r="H28" t="s">
-        <v>158</v>
-      </c>
-      <c r="I28" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="L28" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M28" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N28" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O28" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P28" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q28" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="R28" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="S28" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
       <c r="T28" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
     </row>
     <row r="29" spans="1:20">
@@ -2563,55 +2596,58 @@
         <v>46</v>
       </c>
       <c r="B29" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C29" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D29" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E29" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F29" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G29" s="2">
         <v>45877</v>
       </c>
       <c r="H29" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="I29" t="s">
-        <v>170</v>
+        <v>175</v>
+      </c>
+      <c r="J29" t="s">
+        <v>177</v>
       </c>
       <c r="L29" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M29" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N29" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O29" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P29" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q29" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R29" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="S29" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="T29" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
     </row>
     <row r="30" spans="1:20">
@@ -2619,55 +2655,55 @@
         <v>47</v>
       </c>
       <c r="B30" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C30" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D30" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E30" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F30" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G30" s="2">
         <v>45878</v>
       </c>
       <c r="H30" t="s">
-        <v>160</v>
-      </c>
-      <c r="I30" t="s">
-        <v>170</v>
+        <v>163</v>
+      </c>
+      <c r="J30" t="s">
+        <v>178</v>
       </c>
       <c r="L30" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M30" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N30" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O30" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P30" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q30" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="R30" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="S30" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="T30" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
     </row>
     <row r="31" spans="1:20">
@@ -2675,55 +2711,58 @@
         <v>48</v>
       </c>
       <c r="B31" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C31" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D31" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E31" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F31" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G31" s="2">
         <v>45879</v>
       </c>
       <c r="H31" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="I31" t="s">
-        <v>170</v>
+        <v>171</v>
+      </c>
+      <c r="J31" t="s">
+        <v>176</v>
       </c>
       <c r="L31" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M31" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N31" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O31" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P31" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q31" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="R31" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="S31" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="T31" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
     </row>
     <row r="32" spans="1:20">
@@ -2731,58 +2770,55 @@
         <v>49</v>
       </c>
       <c r="B32" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C32" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D32" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E32" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F32" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G32" s="2">
         <v>45879</v>
       </c>
       <c r="H32" t="s">
-        <v>161</v>
-      </c>
-      <c r="I32" t="s">
-        <v>170</v>
-      </c>
-      <c r="K32" t="s">
-        <v>172</v>
+        <v>164</v>
+      </c>
+      <c r="J32" t="s">
+        <v>176</v>
       </c>
       <c r="L32" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M32" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N32" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O32" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P32" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q32" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R32" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="S32" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="T32" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
     </row>
     <row r="33" spans="1:20">
@@ -2790,58 +2826,55 @@
         <v>49</v>
       </c>
       <c r="B33" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C33" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D33" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E33" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F33" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G33" s="2">
         <v>45879</v>
       </c>
       <c r="H33" t="s">
-        <v>162</v>
-      </c>
-      <c r="I33" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="K33" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="L33" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M33" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N33" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O33" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P33" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q33" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R33" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="S33" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="T33" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
     </row>
     <row r="34" spans="1:20">
@@ -2849,58 +2882,55 @@
         <v>50</v>
       </c>
       <c r="B34" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C34" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D34" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E34" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F34" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G34" s="2">
         <v>45884</v>
       </c>
       <c r="H34" t="s">
-        <v>138</v>
-      </c>
-      <c r="I34" t="s">
-        <v>171</v>
-      </c>
-      <c r="K34" t="s">
-        <v>173</v>
+        <v>141</v>
+      </c>
+      <c r="J34" t="s">
+        <v>177</v>
       </c>
       <c r="L34" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M34" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N34" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O34" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P34" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q34" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R34" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="S34" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="T34" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
     </row>
     <row r="35" spans="1:20">
@@ -2908,58 +2938,55 @@
         <v>50</v>
       </c>
       <c r="B35" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C35" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D35" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E35" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F35" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G35" s="2">
         <v>45884</v>
       </c>
       <c r="H35" t="s">
-        <v>161</v>
-      </c>
-      <c r="I35" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="K35" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="L35" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M35" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N35" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O35" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P35" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q35" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R35" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="S35" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="T35" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
     </row>
     <row r="36" spans="1:20">
@@ -2967,58 +2994,55 @@
         <v>51</v>
       </c>
       <c r="B36" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C36" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D36" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E36" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F36" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G36" s="2">
         <v>45889</v>
       </c>
       <c r="H36" t="s">
-        <v>137</v>
-      </c>
-      <c r="I36" t="s">
-        <v>170</v>
-      </c>
-      <c r="K36" t="s">
-        <v>171</v>
+        <v>140</v>
+      </c>
+      <c r="J36" t="s">
+        <v>178</v>
       </c>
       <c r="L36" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M36" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N36" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O36" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P36" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q36" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R36" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="S36" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="T36" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
     </row>
     <row r="37" spans="1:20">
@@ -3026,58 +3050,55 @@
         <v>51</v>
       </c>
       <c r="B37" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C37" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D37" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E37" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F37" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G37" s="2">
         <v>45889</v>
       </c>
       <c r="H37" t="s">
-        <v>163</v>
-      </c>
-      <c r="I37" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="K37" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="L37" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M37" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N37" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O37" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P37" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q37" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R37" t="s">
-        <v>183</v>
+        <v>196</v>
       </c>
       <c r="S37" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
       <c r="T37" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
     </row>
     <row r="38" spans="1:20">
@@ -3085,58 +3106,55 @@
         <v>51</v>
       </c>
       <c r="B38" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C38" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D38" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E38" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F38" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G38" s="2">
         <v>45889</v>
       </c>
       <c r="H38" t="s">
-        <v>162</v>
-      </c>
-      <c r="I38" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="K38" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="L38" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M38" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N38" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O38" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P38" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q38" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R38" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="S38" t="s">
-        <v>194</v>
+        <v>204</v>
       </c>
       <c r="T38" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
     </row>
     <row r="39" spans="1:20">
@@ -3144,335 +3162,447 @@
         <v>52</v>
       </c>
       <c r="B39" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C39" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D39" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E39" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F39" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G39" s="2">
-        <v>45877</v>
+        <v>45894</v>
       </c>
       <c r="H39" t="s">
-        <v>140</v>
-      </c>
-      <c r="I39" t="s">
-        <v>168</v>
+        <v>151</v>
+      </c>
+      <c r="K39" t="s">
+        <v>176</v>
       </c>
       <c r="L39" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M39" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N39" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O39" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P39" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q39" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R39" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="S39" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="T39" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
     </row>
     <row r="40" spans="1:20">
       <c r="A40" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B40" t="s">
         <v>91</v>
       </c>
       <c r="C40" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D40" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E40" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F40" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G40" s="2">
-        <v>45880</v>
+        <v>45894</v>
       </c>
       <c r="H40" t="s">
-        <v>142</v>
-      </c>
-      <c r="I40" t="s">
-        <v>168</v>
+        <v>141</v>
+      </c>
+      <c r="K40" t="s">
+        <v>176</v>
       </c>
       <c r="L40" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M40" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N40" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O40" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P40" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q40" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R40" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="S40" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="T40" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
     </row>
     <row r="41" spans="1:20">
       <c r="A41" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B41" t="s">
         <v>92</v>
       </c>
       <c r="C41" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D41" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E41" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F41" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G41" s="2">
-        <v>45883</v>
+        <v>45877</v>
       </c>
       <c r="H41" t="s">
-        <v>164</v>
+        <v>143</v>
       </c>
       <c r="I41" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="L41" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M41" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N41" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O41" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P41" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q41" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R41" t="s">
-        <v>186</v>
+        <v>196</v>
       </c>
       <c r="S41" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="T41" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
     </row>
     <row r="42" spans="1:20">
       <c r="A42" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B42" t="s">
         <v>93</v>
       </c>
       <c r="C42" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D42" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E42" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F42" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G42" s="2">
-        <v>45886</v>
+        <v>45880</v>
       </c>
       <c r="H42" t="s">
-        <v>165</v>
+        <v>145</v>
       </c>
       <c r="I42" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="L42" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M42" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N42" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O42" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P42" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q42" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R42" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="S42" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="T42" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
     </row>
     <row r="43" spans="1:20">
       <c r="A43" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B43" t="s">
         <v>94</v>
       </c>
       <c r="C43" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D43" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E43" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F43" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G43" s="2">
-        <v>45889</v>
+        <v>45883</v>
       </c>
       <c r="H43" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I43" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="L43" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="M43" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="N43" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="O43" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="P43" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="Q43" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="R43" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="S43" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="T43" t="s">
-        <v>197</v>
+        <v>207</v>
       </c>
     </row>
     <row r="44" spans="1:20">
       <c r="A44" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B44" t="s">
         <v>95</v>
       </c>
       <c r="C44" t="s">
+        <v>98</v>
+      </c>
+      <c r="D44" t="s">
+        <v>99</v>
+      </c>
+      <c r="E44" t="s">
+        <v>136</v>
+      </c>
+      <c r="F44" t="s">
+        <v>139</v>
+      </c>
+      <c r="G44" s="2">
+        <v>45886</v>
+      </c>
+      <c r="H44" t="s">
+        <v>168</v>
+      </c>
+      <c r="I44" t="s">
+        <v>171</v>
+      </c>
+      <c r="L44" t="s">
+        <v>179</v>
+      </c>
+      <c r="M44" t="s">
+        <v>180</v>
+      </c>
+      <c r="N44" t="s">
+        <v>181</v>
+      </c>
+      <c r="O44" t="s">
+        <v>182</v>
+      </c>
+      <c r="P44" t="s">
+        <v>183</v>
+      </c>
+      <c r="Q44" t="s">
+        <v>184</v>
+      </c>
+      <c r="R44" t="s">
+        <v>197</v>
+      </c>
+      <c r="S44" t="s">
+        <v>204</v>
+      </c>
+      <c r="T44" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="45" spans="1:20">
+      <c r="A45" t="s">
+        <v>57</v>
+      </c>
+      <c r="B45" t="s">
         <v>96</v>
       </c>
-      <c r="D44" t="s">
+      <c r="C45" t="s">
+        <v>98</v>
+      </c>
+      <c r="D45" t="s">
+        <v>99</v>
+      </c>
+      <c r="E45" t="s">
+        <v>137</v>
+      </c>
+      <c r="F45" t="s">
+        <v>139</v>
+      </c>
+      <c r="G45" s="2">
+        <v>45889</v>
+      </c>
+      <c r="H45" t="s">
+        <v>169</v>
+      </c>
+      <c r="I45" t="s">
+        <v>171</v>
+      </c>
+      <c r="L45" t="s">
+        <v>179</v>
+      </c>
+      <c r="M45" t="s">
+        <v>180</v>
+      </c>
+      <c r="N45" t="s">
+        <v>181</v>
+      </c>
+      <c r="O45" t="s">
+        <v>182</v>
+      </c>
+      <c r="P45" t="s">
+        <v>183</v>
+      </c>
+      <c r="Q45" t="s">
+        <v>184</v>
+      </c>
+      <c r="R45" t="s">
+        <v>188</v>
+      </c>
+      <c r="S45" t="s">
+        <v>198</v>
+      </c>
+      <c r="T45" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="46" spans="1:20">
+      <c r="A46" t="s">
+        <v>58</v>
+      </c>
+      <c r="B46" t="s">
         <v>97</v>
       </c>
-      <c r="E44" t="s">
-        <v>135</v>
-      </c>
-      <c r="F44" t="s">
-        <v>136</v>
-      </c>
-      <c r="G44" s="2">
+      <c r="C46" t="s">
+        <v>98</v>
+      </c>
+      <c r="D46" t="s">
+        <v>99</v>
+      </c>
+      <c r="E46" t="s">
+        <v>138</v>
+      </c>
+      <c r="F46" t="s">
+        <v>139</v>
+      </c>
+      <c r="G46" s="2">
         <v>45892</v>
       </c>
-      <c r="H44" t="s">
-        <v>167</v>
-      </c>
-      <c r="I44" t="s">
-        <v>168</v>
-      </c>
-      <c r="L44" t="s">
-        <v>174</v>
-      </c>
-      <c r="M44" t="s">
-        <v>175</v>
-      </c>
-      <c r="N44" t="s">
-        <v>176</v>
-      </c>
-      <c r="O44" t="s">
-        <v>177</v>
-      </c>
-      <c r="P44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q44" t="s">
-        <v>179</v>
-      </c>
-      <c r="R44" t="s">
-        <v>187</v>
-      </c>
-      <c r="S44" t="s">
-        <v>195</v>
-      </c>
-      <c r="T44" t="s">
-        <v>197</v>
+      <c r="H46" t="s">
+        <v>170</v>
+      </c>
+      <c r="I46" t="s">
+        <v>171</v>
+      </c>
+      <c r="L46" t="s">
+        <v>179</v>
+      </c>
+      <c r="M46" t="s">
+        <v>180</v>
+      </c>
+      <c r="N46" t="s">
+        <v>181</v>
+      </c>
+      <c r="O46" t="s">
+        <v>182</v>
+      </c>
+      <c r="P46" t="s">
+        <v>183</v>
+      </c>
+      <c r="Q46" t="s">
+        <v>184</v>
+      </c>
+      <c r="R46" t="s">
+        <v>191</v>
+      </c>
+      <c r="S46" t="s">
+        <v>201</v>
+      </c>
+      <c r="T46" t="s">
+        <v>205</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Melhorias no Frontend - Precisa corrigir o bug de não mostrar as comissões nos casos de CROSS-SELLING
</commit_message>
<xml_diff>
--- a/Faturados.xlsx
+++ b/Faturados.xlsx
@@ -436,13 +436,13 @@
     <t>FATURADO</t>
   </si>
   <si>
-    <t>60000</t>
-  </si>
-  <si>
-    <t>48000</t>
-  </si>
-  <si>
-    <t>150000</t>
+    <t>12000</t>
+  </si>
+  <si>
+    <t>10000</t>
+  </si>
+  <si>
+    <t>16000</t>
   </si>
   <si>
     <t>50000</t>
@@ -460,79 +460,79 @@
     <t>25000</t>
   </si>
   <si>
-    <t>20500</t>
-  </si>
-  <si>
-    <t>21000</t>
-  </si>
-  <si>
-    <t>21500</t>
-  </si>
-  <si>
-    <t>22000</t>
-  </si>
-  <si>
-    <t>22500</t>
-  </si>
-  <si>
-    <t>23000</t>
-  </si>
-  <si>
-    <t>23500</t>
-  </si>
-  <si>
-    <t>24000</t>
-  </si>
-  <si>
-    <t>24500</t>
-  </si>
-  <si>
-    <t>25500</t>
-  </si>
-  <si>
-    <t>26000</t>
-  </si>
-  <si>
-    <t>26500</t>
-  </si>
-  <si>
-    <t>27000</t>
-  </si>
-  <si>
-    <t>27500</t>
+    <t>7400</t>
+  </si>
+  <si>
+    <t>7800</t>
+  </si>
+  <si>
+    <t>8200</t>
+  </si>
+  <si>
+    <t>8600</t>
+  </si>
+  <si>
+    <t>9000</t>
+  </si>
+  <si>
+    <t>9400</t>
+  </si>
+  <si>
+    <t>9800</t>
+  </si>
+  <si>
+    <t>10200</t>
+  </si>
+  <si>
+    <t>10600</t>
+  </si>
+  <si>
+    <t>11000</t>
+  </si>
+  <si>
+    <t>11400</t>
+  </si>
+  <si>
+    <t>11800</t>
+  </si>
+  <si>
+    <t>12200</t>
+  </si>
+  <si>
+    <t>12600</t>
+  </si>
+  <si>
+    <t>13000</t>
+  </si>
+  <si>
+    <t>13400</t>
+  </si>
+  <si>
+    <t>13800</t>
+  </si>
+  <si>
+    <t>14200</t>
+  </si>
+  <si>
+    <t>14600</t>
+  </si>
+  <si>
+    <t>8000</t>
+  </si>
+  <si>
+    <t>5000</t>
+  </si>
+  <si>
+    <t>18000</t>
+  </si>
+  <si>
+    <t>35000</t>
+  </si>
+  <si>
+    <t>40000</t>
   </si>
   <si>
     <t>28000</t>
-  </si>
-  <si>
-    <t>28500</t>
-  </si>
-  <si>
-    <t>29000</t>
-  </si>
-  <si>
-    <t>29500</t>
-  </si>
-  <si>
-    <t>10000</t>
-  </si>
-  <si>
-    <t>8000</t>
-  </si>
-  <si>
-    <t>12000</t>
-  </si>
-  <si>
-    <t>5000</t>
-  </si>
-  <si>
-    <t>18000</t>
-  </si>
-  <si>
-    <t>35000</t>
-  </si>
-  <si>
-    <t>40000</t>
   </si>
   <si>
     <t>32000</t>
@@ -2220,7 +2220,7 @@
         <v>45894</v>
       </c>
       <c r="H21" t="s">
-        <v>147</v>
+        <v>157</v>
       </c>
       <c r="I21" t="s">
         <v>174</v>
@@ -2279,7 +2279,7 @@
         <v>45895</v>
       </c>
       <c r="H22" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="I22" t="s">
         <v>174</v>
@@ -2338,7 +2338,7 @@
         <v>45896</v>
       </c>
       <c r="H23" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I23" t="s">
         <v>176</v>
@@ -2397,7 +2397,7 @@
         <v>45897</v>
       </c>
       <c r="H24" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="I24" t="s">
         <v>177</v>
@@ -2456,7 +2456,7 @@
         <v>45898</v>
       </c>
       <c r="H25" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I25" t="s">
         <v>178</v>
@@ -2515,7 +2515,7 @@
         <v>45874</v>
       </c>
       <c r="H26" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="I26" t="s">
         <v>176</v>
@@ -2574,7 +2574,7 @@
         <v>45875</v>
       </c>
       <c r="H27" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I27" t="s">
         <v>175</v>
@@ -2633,7 +2633,7 @@
         <v>45876</v>
       </c>
       <c r="H28" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="I28" t="s">
         <v>174</v>
@@ -2692,7 +2692,7 @@
         <v>45877</v>
       </c>
       <c r="H29" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="I29" t="s">
         <v>179</v>
@@ -2751,7 +2751,7 @@
         <v>45878</v>
       </c>
       <c r="H30" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I30" t="s">
         <v>177</v>
@@ -2810,7 +2810,7 @@
         <v>45879</v>
       </c>
       <c r="H31" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="I31" t="s">
         <v>174</v>
@@ -2869,7 +2869,7 @@
         <v>45879</v>
       </c>
       <c r="H32" t="s">
-        <v>166</v>
+        <v>141</v>
       </c>
       <c r="I32" t="s">
         <v>178</v>
@@ -2987,7 +2987,7 @@
         <v>45884</v>
       </c>
       <c r="H34" t="s">
-        <v>168</v>
+        <v>140</v>
       </c>
       <c r="I34" t="s">
         <v>175</v>
@@ -3046,7 +3046,7 @@
         <v>45884</v>
       </c>
       <c r="H35" t="s">
-        <v>166</v>
+        <v>141</v>
       </c>
       <c r="I35" t="s">
         <v>174</v>
@@ -3164,7 +3164,7 @@
         <v>45889</v>
       </c>
       <c r="H37" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="I37" t="s">
         <v>176</v>
@@ -3282,7 +3282,7 @@
         <v>45894</v>
       </c>
       <c r="H39" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="I39" t="s">
         <v>175</v>
@@ -3341,7 +3341,7 @@
         <v>45894</v>
       </c>
       <c r="H40" t="s">
-        <v>168</v>
+        <v>140</v>
       </c>
       <c r="I40" t="s">
         <v>175</v>
@@ -3518,7 +3518,7 @@
         <v>45883</v>
       </c>
       <c r="H43" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="I43" t="s">
         <v>174</v>
@@ -3577,7 +3577,7 @@
         <v>45886</v>
       </c>
       <c r="H44" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="I44" t="s">
         <v>174</v>
@@ -3636,7 +3636,7 @@
         <v>45889</v>
       </c>
       <c r="H45" t="s">
-        <v>162</v>
+        <v>172</v>
       </c>
       <c r="I45" t="s">
         <v>174</v>

</xml_diff>